<commit_message>
fix: placar do jogo Jordânia x Argélia feat: backgrounds. atualização do dashboard
</commit_message>
<xml_diff>
--- a/CopadoMundoFIFA2026_DadosPowerBI.xlsx
+++ b/CopadoMundoFIFA2026_DadosPowerBI.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30327"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9018FC1F-37E8-48A7-AE67-7BE5CF9C2266}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D8B8665-F9BC-47A3-B50E-10055E8B3A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="4" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DimSelecao" sheetId="1" r:id="rId1"/>
@@ -11706,7 +11706,7 @@
         <v>577</v>
       </c>
       <c r="I45">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45">
         <v>2</v>

</xml_diff>